<commit_message>
some changes to disk
</commit_message>
<xml_diff>
--- a/evaluations/count/population_counting_results.xlsx
+++ b/evaluations/count/population_counting_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -643,7 +643,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IPanda50</t>
+          <t>HyenaID2022</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -664,13 +664,13 @@
         <v>62500</v>
       </c>
       <c r="G4" t="n">
-        <v>2001</v>
+        <v>3164</v>
       </c>
       <c r="H4" t="n">
-        <v>2001</v>
+        <v>3164</v>
       </c>
       <c r="I4" t="n">
-        <v>338</v>
+        <v>585</v>
       </c>
       <c r="J4" t="b">
         <v>1</v>
@@ -688,15 +688,75 @@
         <v>0</v>
       </c>
       <c r="O4" t="n">
+        <v>1447.59</v>
+      </c>
+      <c r="P4" t="n">
+        <v>85.42</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>169.59</v>
+      </c>
+      <c r="R4" t="n">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>IPanda50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>disk</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>250</v>
+      </c>
+      <c r="D5" t="n">
+        <v>250</v>
+      </c>
+      <c r="E5" t="n">
+        <v>62500</v>
+      </c>
+      <c r="F5" t="n">
+        <v>62500</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2001</v>
+      </c>
+      <c r="I5" t="n">
+        <v>338</v>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" t="n">
+        <v>256</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
         <v>3890.52</v>
       </c>
-      <c r="P4" t="n">
+      <c r="P5" t="n">
         <v>229.84</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="Q5" t="n">
         <v>268.72</v>
       </c>
-      <c r="R4" t="n">
+      <c r="R5" t="n">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete revamp of the evaluation system
</commit_message>
<xml_diff>
--- a/evaluations/count/population_counting_results.xlsx
+++ b/evaluations/count/population_counting_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:S8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,6 +519,11 @@
           <t>Ground Truth</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Mutliscale Enabled</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -579,11 +584,12 @@
       <c r="R2" t="n">
         <v>182</v>
       </c>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BelugaID</t>
+          <t>ATRW</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -592,25 +598,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="D3" t="n">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="E3" t="n">
-        <v>62500</v>
+        <v>2500</v>
       </c>
       <c r="F3" t="n">
-        <v>62500</v>
+        <v>2500</v>
       </c>
       <c r="G3" t="n">
-        <v>4149</v>
+        <v>224</v>
       </c>
       <c r="H3" t="n">
-        <v>4149</v>
+        <v>224</v>
       </c>
       <c r="I3" t="n">
-        <v>306</v>
+        <v>224</v>
       </c>
       <c r="J3" t="b">
         <v>1</v>
@@ -628,22 +634,25 @@
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>4427.59</v>
+        <v>686.37</v>
       </c>
       <c r="P3" t="n">
-        <v>213.39</v>
+        <v>217.23</v>
       </c>
       <c r="Q3" t="n">
-        <v>320.28</v>
+        <v>0.76</v>
       </c>
       <c r="R3" t="n">
-        <v>788</v>
+        <v>182</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HyenaID2022</t>
+          <t>ATRW</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -652,25 +661,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="D4" t="n">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="E4" t="n">
-        <v>62500</v>
+        <v>2500</v>
       </c>
       <c r="F4" t="n">
-        <v>62500</v>
+        <v>2500</v>
       </c>
       <c r="G4" t="n">
-        <v>3164</v>
+        <v>223</v>
       </c>
       <c r="H4" t="n">
-        <v>3164</v>
+        <v>223</v>
       </c>
       <c r="I4" t="n">
-        <v>585</v>
+        <v>223</v>
       </c>
       <c r="J4" t="b">
         <v>1</v>
@@ -688,22 +697,25 @@
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>1447.59</v>
+        <v>962.74</v>
       </c>
       <c r="P4" t="n">
-        <v>85.42</v>
+        <v>276.97</v>
       </c>
       <c r="Q4" t="n">
-        <v>169.59</v>
+        <v>0.76</v>
       </c>
       <c r="R4" t="n">
-        <v>256</v>
+        <v>182</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IPanda50</t>
+          <t>ATRW</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -712,25 +724,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="D5" t="n">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="E5" t="n">
-        <v>62500</v>
+        <v>2500</v>
       </c>
       <c r="F5" t="n">
-        <v>62500</v>
+        <v>2500</v>
       </c>
       <c r="G5" t="n">
-        <v>2001</v>
+        <v>155</v>
       </c>
       <c r="H5" t="n">
-        <v>2001</v>
+        <v>155</v>
       </c>
       <c r="I5" t="n">
-        <v>338</v>
+        <v>155</v>
       </c>
       <c r="J5" t="b">
         <v>1</v>
@@ -748,17 +760,203 @@
         <v>0</v>
       </c>
       <c r="O5" t="n">
+        <v>1157.07</v>
+      </c>
+      <c r="P5" t="n">
+        <v>255.97</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>35.28</v>
+      </c>
+      <c r="R5" t="n">
+        <v>182</v>
+      </c>
+      <c r="S5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BelugaID</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>disk</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>250</v>
+      </c>
+      <c r="D6" t="n">
+        <v>250</v>
+      </c>
+      <c r="E6" t="n">
+        <v>62500</v>
+      </c>
+      <c r="F6" t="n">
+        <v>62500</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4149</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4149</v>
+      </c>
+      <c r="I6" t="n">
+        <v>306</v>
+      </c>
+      <c r="J6" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>256</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>4427.59</v>
+      </c>
+      <c r="P6" t="n">
+        <v>213.39</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>320.28</v>
+      </c>
+      <c r="R6" t="n">
+        <v>788</v>
+      </c>
+      <c r="S6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>HyenaID2022</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>disk</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>250</v>
+      </c>
+      <c r="D7" t="n">
+        <v>250</v>
+      </c>
+      <c r="E7" t="n">
+        <v>62500</v>
+      </c>
+      <c r="F7" t="n">
+        <v>62500</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3164</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3164</v>
+      </c>
+      <c r="I7" t="n">
+        <v>585</v>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>256</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1447.59</v>
+      </c>
+      <c r="P7" t="n">
+        <v>85.42</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>169.59</v>
+      </c>
+      <c r="R7" t="n">
+        <v>256</v>
+      </c>
+      <c r="S7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IPanda50</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>disk</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>250</v>
+      </c>
+      <c r="D8" t="n">
+        <v>250</v>
+      </c>
+      <c r="E8" t="n">
+        <v>62500</v>
+      </c>
+      <c r="F8" t="n">
+        <v>62500</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2001</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2001</v>
+      </c>
+      <c r="I8" t="n">
+        <v>338</v>
+      </c>
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>256</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
         <v>3890.52</v>
       </c>
-      <c r="P5" t="n">
+      <c r="P8" t="n">
         <v>229.84</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="Q8" t="n">
         <v>268.72</v>
       </c>
-      <c r="R5" t="n">
+      <c r="R8" t="n">
         <v>50</v>
       </c>
+      <c r="S8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>